<commit_message>
Birth Reqs Page updates
</commit_message>
<xml_diff>
--- a/docs/v2.0.0/StructureDefinition-VRM-MessageParameters.xlsx
+++ b/docs/v2.0.0/StructureDefinition-VRM-MessageParameters.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="230">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-11T16:10:00-04:00</t>
+    <t>2026-03-24T10:39:59-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -360,6 +360,9 @@
     <t>Parameters.parameter</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t xml:space="preserve">BackboneElement
 </t>
   </si>
@@ -625,7 +628,7 @@
     <t>event_year</t>
   </si>
   <si>
-    <t>DOD_YR or DOB_YR or FDOD_YR event year</t>
+    <t>DOD_YR or IDOB_YR or FDOD_YR event year</t>
   </si>
   <si>
     <t>four digit event year</t>
@@ -1747,7 +1750,7 @@
       </c>
       <c r="E7" s="2"/>
       <c r="F7" t="s" s="2">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="G7" t="s" s="2">
         <v>76</v>
@@ -1762,13 +1765,13 @@
         <v>84</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1807,16 +1810,16 @@
         <v>20</v>
       </c>
       <c r="AB7" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AC7" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD7" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE7" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF7" t="s" s="2">
         <v>111</v>
@@ -1831,7 +1834,7 @@
         <v>20</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>20</v>
@@ -1842,10 +1845,10 @@
     </row>
     <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1868,13 +1871,13 @@
         <v>20</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1925,7 +1928,7 @@
         <v>20</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>75</v>
@@ -1948,14 +1951,14 @@
     </row>
     <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
@@ -1974,16 +1977,16 @@
         <v>20</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -2033,7 +2036,7 @@
         <v>20</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>75</v>
@@ -2045,7 +2048,7 @@
         <v>20</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>20</v>
@@ -2056,14 +2059,14 @@
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
@@ -2082,19 +2085,19 @@
         <v>84</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P10" t="s" s="2">
         <v>20</v>
@@ -2143,7 +2146,7 @@
         <v>20</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>75</v>
@@ -2155,21 +2158,21 @@
         <v>20</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2192,13 +2195,13 @@
         <v>84</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2249,7 +2252,7 @@
         <v>20</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>83</v>
@@ -2272,10 +2275,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2298,13 +2301,13 @@
         <v>84</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2355,7 +2358,7 @@
         <v>20</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>75</v>
@@ -2364,7 +2367,7 @@
         <v>83</v>
       </c>
       <c r="AI12" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ12" t="s" s="2">
         <v>95</v>
@@ -2378,10 +2381,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2404,16 +2407,16 @@
         <v>84</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2463,16 +2466,16 @@
         <v>20</v>
       </c>
       <c r="AF13" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI13" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG13" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH13" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI13" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ13" t="s" s="2">
         <v>20</v>
@@ -2486,10 +2489,10 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2515,13 +2518,13 @@
         <v>77</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
@@ -2571,7 +2574,7 @@
         <v>20</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>75</v>
@@ -2594,20 +2597,20 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>20</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>83</v>
@@ -2622,13 +2625,13 @@
         <v>84</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2691,7 +2694,7 @@
         <v>20</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>20</v>
@@ -2702,10 +2705,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2728,13 +2731,13 @@
         <v>20</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2785,7 +2788,7 @@
         <v>20</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>75</v>
@@ -2808,10 +2811,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2834,13 +2837,13 @@
         <v>20</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2891,7 +2894,7 @@
         <v>20</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>75</v>
@@ -2903,7 +2906,7 @@
         <v>20</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>20</v>
@@ -2914,14 +2917,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -2940,19 +2943,19 @@
         <v>84</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O18" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P18" t="s" s="2">
         <v>20</v>
@@ -3001,7 +3004,7 @@
         <v>20</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>75</v>
@@ -3013,21 +3016,21 @@
         <v>20</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK18" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3050,13 +3053,13 @@
         <v>84</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3068,7 +3071,7 @@
         <v>20</v>
       </c>
       <c r="S19" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="T19" t="s" s="2">
         <v>20</v>
@@ -3107,7 +3110,7 @@
         <v>20</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>83</v>
@@ -3130,10 +3133,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3156,13 +3159,13 @@
         <v>84</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3189,11 +3192,11 @@
         <v>20</v>
       </c>
       <c r="X20" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Y20" s="2"/>
       <c r="Z20" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>20</v>
@@ -3211,7 +3214,7 @@
         <v>20</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>75</v>
@@ -3220,7 +3223,7 @@
         <v>83</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>95</v>
@@ -3234,10 +3237,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3260,16 +3263,16 @@
         <v>84</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -3319,16 +3322,16 @@
         <v>20</v>
       </c>
       <c r="AF21" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI21" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG21" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH21" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI21" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ21" t="s" s="2">
         <v>20</v>
@@ -3342,10 +3345,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3371,13 +3374,13 @@
         <v>20</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -3427,7 +3430,7 @@
         <v>20</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>75</v>
@@ -3450,13 +3453,13 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B23" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D23" t="s" s="2">
         <v>20</v>
@@ -3478,13 +3481,13 @@
         <v>84</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3547,7 +3550,7 @@
         <v>20</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK23" t="s" s="2">
         <v>20</v>
@@ -3558,10 +3561,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3584,13 +3587,13 @@
         <v>20</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3641,7 +3644,7 @@
         <v>20</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>75</v>
@@ -3664,10 +3667,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3690,13 +3693,13 @@
         <v>20</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3747,7 +3750,7 @@
         <v>20</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>75</v>
@@ -3759,7 +3762,7 @@
         <v>20</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>20</v>
@@ -3770,14 +3773,14 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -3796,19 +3799,19 @@
         <v>84</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -3857,7 +3860,7 @@
         <v>20</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>75</v>
@@ -3869,21 +3872,21 @@
         <v>20</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3906,13 +3909,13 @@
         <v>84</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3924,7 +3927,7 @@
         <v>20</v>
       </c>
       <c r="S27" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T27" t="s" s="2">
         <v>20</v>
@@ -3963,7 +3966,7 @@
         <v>20</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>83</v>
@@ -3986,10 +3989,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4012,13 +4015,13 @@
         <v>84</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4069,7 +4072,7 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>75</v>
@@ -4078,7 +4081,7 @@
         <v>83</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ28" t="s" s="2">
         <v>95</v>
@@ -4092,10 +4095,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4118,16 +4121,16 @@
         <v>84</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4177,16 +4180,16 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI29" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG29" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ29" t="s" s="2">
         <v>20</v>
@@ -4200,10 +4203,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4229,13 +4232,13 @@
         <v>20</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4285,7 +4288,7 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>75</v>
@@ -4308,13 +4311,13 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B31" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D31" t="s" s="2">
         <v>20</v>
@@ -4336,13 +4339,13 @@
         <v>84</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4405,7 +4408,7 @@
         <v>20</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>20</v>
@@ -4416,10 +4419,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4442,13 +4445,13 @@
         <v>20</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4499,7 +4502,7 @@
         <v>20</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>75</v>
@@ -4522,10 +4525,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4548,13 +4551,13 @@
         <v>20</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4605,7 +4608,7 @@
         <v>20</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>75</v>
@@ -4617,7 +4620,7 @@
         <v>20</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>20</v>
@@ -4628,14 +4631,14 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -4654,19 +4657,19 @@
         <v>84</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>20</v>
@@ -4715,7 +4718,7 @@
         <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>75</v>
@@ -4727,21 +4730,21 @@
         <v>20</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4764,13 +4767,13 @@
         <v>84</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4782,7 +4785,7 @@
         <v>20</v>
       </c>
       <c r="S35" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="T35" t="s" s="2">
         <v>20</v>
@@ -4821,7 +4824,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>83</v>
@@ -4844,10 +4847,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4870,13 +4873,13 @@
         <v>84</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4927,7 +4930,7 @@
         <v>20</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>75</v>
@@ -4936,7 +4939,7 @@
         <v>83</v>
       </c>
       <c r="AI36" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ36" t="s" s="2">
         <v>95</v>
@@ -4950,10 +4953,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -4976,16 +4979,16 @@
         <v>84</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5035,16 +5038,16 @@
         <v>20</v>
       </c>
       <c r="AF37" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG37" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH37" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI37" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG37" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH37" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI37" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>20</v>
@@ -5058,10 +5061,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5087,13 +5090,13 @@
         <v>20</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -5143,7 +5146,7 @@
         <v>20</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>75</v>
@@ -5166,13 +5169,13 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B39" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D39" t="s" s="2">
         <v>20</v>
@@ -5194,13 +5197,13 @@
         <v>84</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5263,7 +5266,7 @@
         <v>20</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>20</v>
@@ -5274,10 +5277,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5300,13 +5303,13 @@
         <v>20</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5357,7 +5360,7 @@
         <v>20</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>75</v>
@@ -5380,10 +5383,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5406,13 +5409,13 @@
         <v>20</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5463,7 +5466,7 @@
         <v>20</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>75</v>
@@ -5475,7 +5478,7 @@
         <v>20</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>20</v>
@@ -5486,14 +5489,14 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -5512,19 +5515,19 @@
         <v>84</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>20</v>
@@ -5573,7 +5576,7 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>75</v>
@@ -5585,21 +5588,21 @@
         <v>20</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -5622,13 +5625,13 @@
         <v>84</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -5640,7 +5643,7 @@
         <v>20</v>
       </c>
       <c r="S43" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="T43" t="s" s="2">
         <v>20</v>
@@ -5679,7 +5682,7 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>83</v>
@@ -5702,10 +5705,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -5728,13 +5731,13 @@
         <v>84</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -5785,7 +5788,7 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>75</v>
@@ -5794,7 +5797,7 @@
         <v>83</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>95</v>
@@ -5808,10 +5811,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -5834,16 +5837,16 @@
         <v>84</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -5893,16 +5896,16 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI45" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG45" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH45" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI45" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>20</v>
@@ -5916,10 +5919,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -5945,13 +5948,13 @@
         <v>20</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6001,7 +6004,7 @@
         <v>20</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>75</v>
@@ -6024,13 +6027,13 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B47" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D47" t="s" s="2">
         <v>20</v>
@@ -6052,13 +6055,13 @@
         <v>84</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -6121,7 +6124,7 @@
         <v>20</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK47" t="s" s="2">
         <v>20</v>
@@ -6132,10 +6135,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6158,13 +6161,13 @@
         <v>20</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -6215,7 +6218,7 @@
         <v>20</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>75</v>
@@ -6238,10 +6241,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6264,13 +6267,13 @@
         <v>20</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -6321,7 +6324,7 @@
         <v>20</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>75</v>
@@ -6333,7 +6336,7 @@
         <v>20</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>20</v>
@@ -6344,14 +6347,14 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
@@ -6370,19 +6373,19 @@
         <v>84</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O50" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>20</v>
@@ -6431,7 +6434,7 @@
         <v>20</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>75</v>
@@ -6443,21 +6446,21 @@
         <v>20</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK50" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6480,13 +6483,13 @@
         <v>84</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -6498,7 +6501,7 @@
         <v>20</v>
       </c>
       <c r="S51" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="T51" t="s" s="2">
         <v>20</v>
@@ -6537,7 +6540,7 @@
         <v>20</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -6560,10 +6563,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -6586,13 +6589,13 @@
         <v>84</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -6643,7 +6646,7 @@
         <v>20</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>75</v>
@@ -6652,7 +6655,7 @@
         <v>83</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ52" t="s" s="2">
         <v>95</v>
@@ -6666,10 +6669,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6692,16 +6695,16 @@
         <v>84</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -6751,16 +6754,16 @@
         <v>20</v>
       </c>
       <c r="AF53" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI53" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ53" t="s" s="2">
         <v>20</v>
@@ -6774,10 +6777,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -6803,13 +6806,13 @@
         <v>20</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -6859,7 +6862,7 @@
         <v>20</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>75</v>
@@ -6882,13 +6885,13 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B55" t="s" s="2">
         <v>111</v>
       </c>
       <c r="C55" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D55" t="s" s="2">
         <v>20</v>
@@ -6910,13 +6913,13 @@
         <v>84</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -6979,7 +6982,7 @@
         <v>20</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>20</v>
@@ -6990,10 +6993,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -7016,13 +7019,13 @@
         <v>20</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -7073,7 +7076,7 @@
         <v>20</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>75</v>
@@ -7096,10 +7099,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -7122,13 +7125,13 @@
         <v>20</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -7179,7 +7182,7 @@
         <v>20</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>75</v>
@@ -7191,7 +7194,7 @@
         <v>20</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK57" t="s" s="2">
         <v>20</v>
@@ -7202,14 +7205,14 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
@@ -7228,19 +7231,19 @@
         <v>84</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O58" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>20</v>
@@ -7289,7 +7292,7 @@
         <v>20</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>75</v>
@@ -7301,21 +7304,21 @@
         <v>20</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7338,13 +7341,13 @@
         <v>84</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -7356,7 +7359,7 @@
         <v>20</v>
       </c>
       <c r="S59" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="T59" t="s" s="2">
         <v>20</v>
@@ -7395,7 +7398,7 @@
         <v>20</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>83</v>
@@ -7418,10 +7421,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7444,13 +7447,13 @@
         <v>84</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -7477,11 +7480,11 @@
         <v>20</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y60" s="2"/>
       <c r="Z60" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>20</v>
@@ -7499,7 +7502,7 @@
         <v>20</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>75</v>
@@ -7508,7 +7511,7 @@
         <v>83</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AJ60" t="s" s="2">
         <v>95</v>
@@ -7522,10 +7525,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -7548,16 +7551,16 @@
         <v>84</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -7607,16 +7610,16 @@
         <v>20</v>
       </c>
       <c r="AF61" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="AG61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AH61" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI61" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="AG61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH61" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI61" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AJ61" t="s" s="2">
         <v>20</v>
@@ -7630,10 +7633,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -7659,13 +7662,13 @@
         <v>20</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -7715,7 +7718,7 @@
         <v>20</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>75</v>

</xml_diff>